<commit_message>
upto 24-07-2025 changes moving
</commit_message>
<xml_diff>
--- a/STA UAT/STA Yoga/Templates/UpdatedBulkEmailInwardTemp.xlsx
+++ b/STA UAT/STA Yoga/Templates/UpdatedBulkEmailInwardTemp.xlsx
@@ -13,6 +13,7 @@
   </bookViews>
   <sheets>
     <sheet name="Inward1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Inward1!#REF!</definedName>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="30">
   <si>
     <t>SL NO</t>
   </si>
@@ -114,6 +115,9 @@
   </si>
   <si>
     <t xml:space="preserve">I Forget My Folio No </t>
+  </si>
+  <si>
+    <t>6380611603</t>
   </si>
 </sst>
 </file>
@@ -450,6 +454,121 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.90625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="60.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="76.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="18.6328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="4">
+        <v>45748</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="OT" sqref="C2"/>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -537,7 +656,9 @@
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="H2" s="3" t="s">
+        <v>29</v>
+      </c>
       <c r="I2" s="2" t="s">
         <v>13</v>
       </c>
@@ -621,6 +742,5 @@
     <hyperlink ref="I4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>